<commit_message>
Finalize IRB protocol and data privacy safeguards
</commit_message>
<xml_diff>
--- a/irb_submission/IRB_SUBMISSION_BUNDLE/03_SORA_Electronic_Data_Submission_Template.xlsx
+++ b/irb_submission/IRB_SUBMISSION_BUNDLE/03_SORA_Electronic_Data_Submission_Template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Entry" sheetId="1" r:id="R92ecf88bc42343e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R563e1ce891b44394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Summary" sheetId="3" r:id="R2f881b4ea8214977"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Entry" sheetId="1" r:id="R61091b71b4c34e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R268efd854e0d46ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Summary" sheetId="3" r:id="Rf8eeec418a0844e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4139,7 +4139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c89ea5b32ba458a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7491f89b725848e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4176,12 +4176,12 @@
         <x:v>Enter one eligible patient per row. Do not add columns.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="37" t="str">
         <x:v>site_code</x:v>
       </x:c>
       <x:c r="B5" s="38" t="str">
-        <x:v>Use the nonidentifying site code assigned for this study (for example, SITE01). Do not enter the clinic name.</x:v>
+        <x:v>Use the study site code assigned for analysis (for example, SITE01). Do not enter the clinic name; the clinic-code mapping is stored separately with restricted access.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>